<commit_message>
Wave 1 complete: generator, statements/rules/ratios/verifier, frontend screens
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/seed/portfolio/L-2025-0233/vypiska_2026-07_08.xlsx
+++ b/data/seed/portfolio/L-2025-0233/vypiska_2026-07_08.xlsx
@@ -560,31 +560,31 @@
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n">
-        <v>76369000</v>
+        <v>7197000</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Xiva Poligraf MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>345170902</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>20208000851157093001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №58/26 от 01.07.2026</t>
+          <t>Оплата по с/ф №9024 за поставленный товар</t>
         </is>
       </c>
     </row>
@@ -599,40 +599,40 @@
           <t>101</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n">
-        <v>22445000</v>
-      </c>
+      <c r="C11" s="2" t="n">
+        <v>17253000</v>
+      </c>
+      <c r="D11" s="2" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Navro'z Dori-Darmon MChJ</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>212520987</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000692292337001</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Оплата по с/ф №9676 за поставленный товар</t>
+          <t>Предоплата за материалы по договору №111/26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03.07.2026</t>
+          <t>02.07.2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -640,40 +640,40 @@
           <t>102</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
-        <v>30313000</v>
-      </c>
-      <c r="D12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n">
+        <v>4819000</v>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно счет-фактуре №1243</t>
+          <t>Оплата за продукцию по дог. №195/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05.07.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -681,35 +681,40 @@
           <t>103</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
-        <v>62800000</v>
-      </c>
-      <c r="D13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n">
+        <v>42194000</v>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Kreditni qaytarish hisobvarag'i (L-2025-0233)</t>
+          <t>Sharq Qurilish MChJ</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>16307000237259787417</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Kredit shartnomasi L-2025-0233 bo'yicha navbatdagi to'lov (07.2026)</t>
+          <t>Оплата по счет-фактуре №7538 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06.07.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -719,38 +724,38 @@
       </c>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n">
-        <v>21377000</v>
+        <v>24533000</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oydin Avto Savdo AJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>308210196</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>20208000469112014001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>SHARTNOMA №61/26 BO'YICHA OLDINDAN TO'LOV</t>
+          <t>Оплата за продукцию по дог. №275/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06.07.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -760,21 +765,21 @@
       </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n">
-        <v>5145000</v>
+        <v>5319000</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -784,14 +789,14 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №6710 за поставленный товар</t>
+          <t>Оплата за продукцию по договору №220/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06.07.2026</t>
+          <t>03.07.2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -799,40 +804,40 @@
           <t>106</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
-        <v>21310000</v>
-      </c>
-      <c r="D16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n">
+        <v>2605000</v>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно счет-фактуре №3926</t>
+          <t>Tovar uchun to'lov, hisob-faktura №3298 03.07.2026, QQS bilan</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06.07.2026</t>
+          <t>05.07.2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -841,17 +846,17 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>21809000</v>
+        <v>62800000</v>
       </c>
       <c r="D17" s="2" t="n"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oqsaroy Bank ATB</t>
+          <t>Kreditni qaytarish hisobvarag'i (L-2025-0233)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>45994000900000001001</t>
+          <t>16307000237259787417</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -861,14 +866,14 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Заработная плата за июнь 2026 г. (перечисление на пластиковые карты)</t>
+          <t>Kredit shartnomasi L-2025-0233 bo'yicha navbatdagi to'lov (07.2026)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -876,40 +881,40 @@
           <t>108</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
-        <v>3447000</v>
-      </c>
-      <c r="D18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n">
+        <v>12302000</v>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Navro'z Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>325978388</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>20208000844795834001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Арендная плата за июль 2026 г. по дог. №58/25</t>
+          <t>Предоплата за товар по договору №50/26 от 06.07.2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -917,40 +922,40 @@
           <t>109</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
-        <v>6766000</v>
-      </c>
-      <c r="D19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n">
+        <v>12157000</v>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно счет-фактуре №8173</t>
+          <t>Предоплата за товар по договору №108/26 от 06.07.2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -958,40 +963,40 @@
           <t>110</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n">
-        <v>21205000</v>
-      </c>
-      <c r="D20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n">
+        <v>9374000</v>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №296/26</t>
+          <t>Оплата за товар по с/ф №9059 от 06.07.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -999,23 +1004,23 @@
           <t>111</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n">
-        <v>23375000</v>
-      </c>
-      <c r="D21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n">
+        <v>8546000</v>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Denov Farm Savdo XK</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>278353466</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000791540008001</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1025,14 +1030,14 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Xom ashyo uchun to'lov, shartnoma №77/26, QQS bilan</t>
+          <t>Оплата за продукцию по договору №121/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1042,21 +1047,21 @@
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n">
-        <v>27064000</v>
+        <v>6223000</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Zafar Qurilish XK</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>219004151</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000492719663001</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1066,14 +1071,14 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ОПЛАТА ЗА ТОВАР ПО СЧЕТ-ФАКТУРЕ №5036 ОТ 13.07.2026, В Т.Ч. НДС 12%</t>
+          <t>Оплата за товар по счет-фактуре №6992 от 06.07.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1081,40 +1086,40 @@
           <t>113</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n">
-        <v>15125000</v>
-      </c>
-      <c r="D23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n">
+        <v>2476000</v>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные матеиалы, с/ф №7967</t>
+          <t>Оплата за продукцию по договору №1/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>15.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1122,23 +1127,23 @@
           <t>114</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n">
-        <v>67436000</v>
-      </c>
+      <c r="C24" s="2" t="n">
+        <v>21002000</v>
+      </c>
+      <c r="D24" s="2" t="n"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Xiva Poligraf MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>345170902</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>20208000851157093001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1148,14 +1153,14 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №189/26 от 15.07.2026</t>
+          <t>Оплата за сырье по договору №25/26 от 06.07.2026, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>15.07.2026</t>
+          <t>06.07.2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1164,39 +1169,34 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2974000</v>
+        <v>21809000</v>
       </c>
       <c r="D25" s="2" t="n"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>201122905</t>
+          <t>Oqsaroy Bank ATB</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>45994000900000001001</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Iyun oyi uchun ijtimoiy soliq</t>
+          <t>Заработная плата за июнь 2026 г. (перечисление на пластиковые карты)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>15.07.2026</t>
+          <t>08.07.2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1204,40 +1204,40 @@
           <t>116</t>
         </is>
       </c>
-      <c r="C26" s="2" t="n">
-        <v>2974000</v>
-      </c>
-      <c r="D26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n">
+        <v>3156000</v>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>201122905</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Налог на доходы физических лиц за июнь 2026 г.</t>
+          <t>Оплата за товар по счет-фактуре №3993 от 08.07.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>09.07.2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1247,38 +1247,38 @@
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n">
-        <v>23946000</v>
+        <v>16148000</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Xiva Poligraf MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>345170902</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>20208000851157093001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Mahsulot uchun to'lov, shartn. №266/26, QQS 12%</t>
+          <t>Mahsulot uchun to'lov, shartnoma №156/26, QQS 12%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>09.07.2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1288,21 +1288,21 @@
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n">
-        <v>9599000</v>
+        <v>5366000</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1312,14 +1312,14 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №9785 от 20.07.2026, в т.ч. НДС 12%</t>
+          <t>Shartnoma №233/26 bo'yicha oldindan to'lov</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>09.07.2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1327,40 +1327,40 @@
           <t>119</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n">
-        <v>8365000</v>
-      </c>
+      <c r="C29" s="2" t="n">
+        <v>3447000</v>
+      </c>
+      <c r="D29" s="2" t="n"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Bunyodkor Qurilish MChJ</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>247354122</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000393004688001</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №7604 за поставленный товар</t>
+          <t>Арендная плата за июль 2026 г. по договору №51/25</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>09.07.2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1369,39 +1369,39 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>12015000</v>
+        <v>42652000</v>
       </c>
       <c r="D30" s="2" t="n"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №3871</t>
+          <t>Оплата за упаковочные материалы, с/ф №9266</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>20.07.2026</t>
+          <t>10.07.2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1409,23 +1409,23 @@
           <t>121</t>
         </is>
       </c>
-      <c r="C31" s="2" t="n">
-        <v>69239000</v>
-      </c>
-      <c r="D31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n">
+        <v>3827000</v>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1435,14 +1435,14 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №296/26</t>
+          <t>Оплата по с/ф №5068 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>21.07.2026</t>
+          <t>10.07.2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1450,40 +1450,40 @@
           <t>122</t>
         </is>
       </c>
-      <c r="C32" s="2" t="n">
-        <v>9355000</v>
-      </c>
-      <c r="D32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n">
+        <v>3317000</v>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Shodlik Polimer AJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>322574503</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>20208000927723213001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №4234</t>
+          <t>Оплата за товар по счет-фактуре №6774 от 10.07.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>22.07.2026</t>
+          <t>13.07.2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1491,23 +1491,23 @@
           <t>123</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n">
-        <v>35657000</v>
-      </c>
-      <c r="D33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n">
+        <v>5846000</v>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1517,14 +1517,14 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Оплата за сырье по договору №118/26 от 22.07.2026, НДС 12%</t>
+          <t>Оплата за продукцию по договору №108/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>13.07.2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1532,40 +1532,40 @@
           <t>124</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n">
-        <v>43926000</v>
-      </c>
+      <c r="C34" s="2" t="n">
+        <v>14517000</v>
+      </c>
+      <c r="D34" s="2" t="n"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Xiva Poligraf MChJ</t>
+          <t>Qarshi Un Mahsulotlari MChJ</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>345170902</t>
+          <t>278320484</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>20208000851157093001</t>
+          <t>20208000799048289001</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по договору №12/26, НДС 12%</t>
+          <t>Оплата за сырье по договору №51/26 от 13.07.2026, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>14.07.2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1575,21 +1575,21 @@
       </c>
       <c r="C35" s="2" t="n"/>
       <c r="D35" s="2" t="n">
-        <v>6978000</v>
+        <v>3752000</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Shartnoma №8/26 bo'yicha oldindan to'lov</t>
+          <t>Предоплата за товар по договору №48/26 от 14.07.2026</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>15.07.2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1614,40 +1614,40 @@
           <t>126</t>
         </is>
       </c>
-      <c r="C36" s="2" t="n">
-        <v>5618000</v>
-      </c>
-      <c r="D36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n">
+        <v>10145000</v>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>201122905</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>QQS iyun 2026 uchun</t>
+          <t>Предоплата за товар по договору №58/26 от 15.07.2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>15.07.2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1655,40 +1655,40 @@
           <t>127</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n">
-        <v>6940000</v>
-      </c>
-      <c r="D37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n">
+        <v>10055000</v>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Sharq Qurilish MChJ</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Оплата за срье по дог. №75/26 от 23.07.2026, НДС 12%</t>
+          <t>Shartnoma №100/26 bo'yicha oldindan to'lov</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>15.07.2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1697,39 +1697,39 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>11276000</v>
+        <v>2974000</v>
       </c>
       <c r="D38" s="2" t="n"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Xom ashyo uchun to'lov, shartn. №66/26, QQS bilan</t>
+          <t>Социальный налог за июнь 2026 г.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>15.07.2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1738,39 +1738,39 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>13883000</v>
+        <v>2974000</v>
       </c>
       <c r="D39" s="2" t="n"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №9411</t>
+          <t>НДФЛ за июнь 2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>24.07.2026</t>
+          <t>16.07.2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1778,40 +1778,40 @@
           <t>130</t>
         </is>
       </c>
-      <c r="C40" s="2" t="n">
-        <v>2154000</v>
-      </c>
-      <c r="D40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n">
+        <v>6066000</v>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hududiy elektr tarmoqlari AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>200933985</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>20208000147014124001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Оплата за электроэнергию согласно счету</t>
+          <t>Yetkazilgan tovar uchun to'lov h/f №1341</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>24.07.2026</t>
+          <t>17.07.2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1819,40 +1819,40 @@
           <t>131</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n">
-        <v>11888000</v>
-      </c>
-      <c r="D41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n">
+        <v>31500000</v>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно с/ф №6289</t>
+          <t>Оплата за продукцию по договору №23/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>27.07.2026</t>
+          <t>17.07.2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1862,38 +1862,38 @@
       </c>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n">
-        <v>56053000</v>
+        <v>5966000</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Оплата за товар по с/ф №8887 от 27.07.2026, в т.ч. НДС 12%</t>
+          <t>Оплата за продукцию по договору №292/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>27.07.2026</t>
+          <t>20.07.2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1901,40 +1901,40 @@
           <t>133</t>
         </is>
       </c>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n">
-        <v>6614000</v>
-      </c>
+      <c r="C43" s="2" t="n">
+        <v>13343000</v>
+      </c>
+      <c r="D43" s="2" t="n"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Samarqand Qurilish MChJ</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>378388884</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000795834914001</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00987</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №5294 от 27.07.2026, в т.ч. НДС 12%</t>
+          <t>Оплата за товары согласно счет-фактуре №1281</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>27.07.2026</t>
+          <t>20.07.2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1943,39 +1943,39 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>24292000</v>
+        <v>26788000</v>
       </c>
       <c r="D44" s="2" t="n"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Mehnat Polimer MChJ</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>305873968</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000941692404001</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно с/ф №2342</t>
+          <t>ОПЛАТА ЗА ТРАНСПОРТНЫЕ УСЛУГИ ПО ДОГОВОРУ №134/26</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>28.07.2026</t>
+          <t>20.07.2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1983,40 +1983,40 @@
           <t>135</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n">
-        <v>9311000</v>
-      </c>
+      <c r="C45" s="2" t="n">
+        <v>72025000</v>
+      </c>
+      <c r="D45" s="2" t="n"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ziyo Plastik MChJ</t>
+          <t>Mehnat Polimer MChJ</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>271190041</t>
+          <t>305873968</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>20208000164927196001</t>
+          <t>20208000941692404001</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>MAHSULOT UCHUN TO'LOV, SHARTNOMA №95/26, QQS 12%</t>
+          <t>Оплата за упаковочные материалы, с/ф №2141</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>20.07.2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2024,23 +2024,23 @@
           <t>136</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n">
-        <v>56429000</v>
-      </c>
+      <c r="C46" s="2" t="n">
+        <v>214447000</v>
+      </c>
+      <c r="D46" s="2" t="n"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Farg'ona Poligraf MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>216346862</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>20208000098714257001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2050,14 +2050,14 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №7344 от 29.07.2026, в т.ч. НДС 12%</t>
+          <t>Оплата за сырье по дог. №123/26 от 20.07.2026, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>29.07.2026</t>
+          <t>21.07.2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2065,40 +2065,40 @@
           <t>137</t>
         </is>
       </c>
-      <c r="C47" s="2" t="n">
-        <v>8271000</v>
-      </c>
-      <c r="D47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n">
+        <v>33670000</v>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Shodlik Polimer AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>322574503</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>20208000927723213001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Предоплата за материалы по договору №101/26</t>
+          <t>Оплата за товар по счет-фактуре №8227 от 21.07.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>31.07.2026</t>
+          <t>21.07.2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2108,38 +2108,38 @@
       </c>
       <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n">
-        <v>13896000</v>
+        <v>22411000</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Oqtosh Qog'oz AJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>371514300</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>20208000665316781001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №126/26 от 31.07.2026</t>
+          <t>Оплата по счет-фактуре №9807 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>31.07.2026</t>
+          <t>21.07.2026</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2149,21 +2149,21 @@
       </c>
       <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n">
-        <v>13250000</v>
+        <v>3292000</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2173,14 +2173,14 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №1837 за поставленный товар</t>
+          <t>Оплата за продукцию по договору №47/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>31.07.2026</t>
+          <t>22.07.2026</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2188,35 +2188,40 @@
           <t>140</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n">
+        <v>8504000</v>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Oqsaroy Bank ATB</t>
+          <t>Lazzat Tur Servis MChJ</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>365378468</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>45994000900000001001</t>
+          <t>20208000774037432001</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Комиссия банка за расчетно-кассовое обслуживание за июль</t>
+          <t>Оплата за продукцию о договору №271/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>31.07.2026</t>
+          <t>22.07.2026</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2225,39 +2230,39 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>78550000</v>
+        <v>5814000</v>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №3306</t>
+          <t>Уплата налога на добавленную стоимость за июнь</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>23.07.2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2267,38 +2272,38 @@
       </c>
       <c r="C52" s="2" t="n"/>
       <c r="D52" s="2" t="n">
-        <v>109338000</v>
+        <v>4768000</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по договору №5/26, НДС 12%</t>
+          <t>Оплата за продукцию по договору №81/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>23.07.2026</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2308,38 +2313,38 @@
       </c>
       <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="n">
-        <v>2224000</v>
+        <v>2783000</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Qarshi Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>238804395</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>20208000372184603001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №3216 от 03.08.2026, в т.ч. НДС 12%</t>
+          <t>Mahsulot uchun to'lov, shartn. №57/26, QQS 12%</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>24.07.2026</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2347,40 +2352,40 @@
           <t>144</t>
         </is>
       </c>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n">
-        <v>2219000</v>
-      </c>
+      <c r="C54" s="2" t="n">
+        <v>2154000</v>
+      </c>
+      <c r="D54" s="2" t="n"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Hududiy elektr tarmoqlari AJ</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>200933985</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000028408911001</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №7510 от 03.08.2026, в т.ч. НДС 12%</t>
+          <t>ОПЛАТА ЗА ЭЛЕКТРОЭНЕРГИЮ СОГЛАСНО СЧЕТУ</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>27.07.2026</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2388,40 +2393,40 @@
           <t>145</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n">
-        <v>6953000</v>
-      </c>
-      <c r="D55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n">
+        <v>27768000</v>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Xiva Meva-Sabzavot MChJ</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>257450339</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000772321336001</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Оплата за сырье по договору №84/26 от 03.08.2026, НДС 12%</t>
+          <t>Оплата по с/ф №1205 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>27.07.2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2429,40 +2434,40 @@
           <t>146</t>
         </is>
       </c>
-      <c r="C56" s="2" t="n">
-        <v>7639000</v>
-      </c>
-      <c r="D56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n">
+        <v>9629000</v>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Gulshan Qurilish Materiallari AJ</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>250436474</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000679511638001</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №6/26</t>
+          <t>ОПЛАТА ЗА ПРОДУКЦИЮ ПО ДОГОВОРУ №294/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>03.08.2026</t>
+          <t>27.07.2026</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2470,40 +2475,40 @@
           <t>147</t>
         </is>
       </c>
-      <c r="C57" s="2" t="n">
-        <v>10953000</v>
-      </c>
-      <c r="D57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n">
+        <v>3452000</v>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно счет-фактуре №4610</t>
+          <t>Mahsulot uchun to'lov, shartnoma №249/26, QQS 12%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>04.08.2026</t>
+          <t>27.07.2026</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2511,35 +2516,40 @@
           <t>148</t>
         </is>
       </c>
-      <c r="C58" s="2" t="n">
-        <v>21924000</v>
-      </c>
-      <c r="D58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n">
+        <v>2631000</v>
+      </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Oqsaroy Bank ATB</t>
+          <t>Sharq Qurilish MChJ</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>45994000900000001001</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Перечисление заработной платы за июль 2026 г. согласно реестру №4533</t>
+          <t>Предоплата за товар по договору №215/26 от 27.07.2026</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>05.08.2026</t>
+          <t>28.07.2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2549,38 +2559,38 @@
       </c>
       <c r="C59" s="2" t="n"/>
       <c r="D59" s="2" t="n">
-        <v>2252000</v>
+        <v>5568000</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Denov Farm Savdo XK</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>278353466</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000791540008001</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00987</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №278/26 от 05.08.2026</t>
+          <t>ПРЕДОПЛАТА ЗА ТОВАР ПО ДОГОВОРУ №245/26 ОТ 28.07.2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>05.08.2026</t>
+          <t>28.07.2026</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2590,38 +2600,38 @@
       </c>
       <c r="C60" s="2" t="n"/>
       <c r="D60" s="2" t="n">
-        <v>2017000</v>
+        <v>5003000</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Ziyo Plastik MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>271190041</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>20208000164927196001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Shartnoma №268/26 bo'yicha oldindan to'lov</t>
+          <t>Оплата по счет-фактуре №6285 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>05.08.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2629,40 +2639,40 @@
           <t>151</t>
         </is>
       </c>
-      <c r="C61" s="2" t="n">
-        <v>46735000</v>
-      </c>
-      <c r="D61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n">
+        <v>70227000</v>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Предоплата за материалы по договору №296/26</t>
+          <t>Оплата за продукцию по договору №49/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>05.08.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2670,35 +2680,40 @@
           <t>152</t>
         </is>
       </c>
-      <c r="C62" s="2" t="n">
-        <v>62800000</v>
-      </c>
-      <c r="D62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n">
+        <v>18828000</v>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Kreditni qaytarish hisobvarag'i (L-2025-0233)</t>
+          <t>Xiva Mehmonxona MChJ</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>16307000237259787417</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Kredit shartnomasi L-2025-0233 bo'yicha navbatdagi to'lov (08.2026)</t>
+          <t>ПРЕДОПЛАТА ЗА ТОВАР ПО ДОГ. №30/26 ОТ 29.07.2026</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06.08.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2708,38 +2723,38 @@
       </c>
       <c r="C63" s="2" t="n"/>
       <c r="D63" s="2" t="n">
-        <v>6012000</v>
+        <v>8665000</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Оплата по с/ф №7968 за поставленный товар</t>
+          <t>Yetkazilgan tovar uchun to'lov h/f №4731</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06.08.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2747,40 +2762,40 @@
           <t>154</t>
         </is>
       </c>
-      <c r="C64" s="2" t="n">
-        <v>17843000</v>
-      </c>
-      <c r="D64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n">
+        <v>6717000</v>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Sharq Qurilish MChJ</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №101/26</t>
+          <t>Оплата по счет-фактуре №1389 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>29.07.2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2790,21 +2805,21 @@
       </c>
       <c r="C65" s="2" t="n"/>
       <c r="D65" s="2" t="n">
-        <v>11299000</v>
+        <v>3169000</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2814,14 +2829,14 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №7914 за поставленный товар</t>
+          <t>ПРЕДОПЛАТА ЗА ТОВАР ПО ДОГОВОРУ №9/26 ОТ 29.07.2026</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>30.07.2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2831,38 +2846,38 @@
       </c>
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n">
-        <v>3578000</v>
+        <v>4522000</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Oqtosh Qog'oz AJ</t>
+          <t>Sharq Qurilish MChJ</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>371514300</t>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>20208000665316781001</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №205/26 от 10.08.2026</t>
+          <t>Предоплата за товар по дог. №275/26 от 30.07.2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>31.07.2026</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2870,40 +2885,35 @@
           <t>157</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n">
-        <v>2922000</v>
-      </c>
+      <c r="C67" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D67" s="2" t="n"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>338466336</t>
+          <t>Oqsaroy Bank ATB</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>45994000900000001001</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по дог. №38/26, НДС 12%</t>
+          <t>Комиссия за перевод</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2911,40 +2921,40 @@
           <t>158</t>
         </is>
       </c>
-      <c r="C68" s="2" t="n">
-        <v>3465000</v>
-      </c>
-      <c r="D68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n">
+        <v>48282000</v>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Navro'z Qurilish Materiallari MChJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>325978388</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>20208000844795834001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Аренда помещения за август, дог. №58/25</t>
+          <t>Предоплата за товар по дог. №282/26 от 03.08.2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2952,40 +2962,40 @@
           <t>159</t>
         </is>
       </c>
-      <c r="C69" s="2" t="n">
-        <v>8831000</v>
-      </c>
-      <c r="D69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n">
+        <v>38407000</v>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №70/26</t>
+          <t>Предоплата за товар по договору №29/26 от 03.08.2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>10.08.2026</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2993,40 +3003,40 @@
           <t>160</t>
         </is>
       </c>
-      <c r="C70" s="2" t="n">
-        <v>31882000</v>
-      </c>
-      <c r="D70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n">
+        <v>20526000</v>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Предоплата за материалы по договору №141/26</t>
+          <t>ОПЛАТА ПО С/Ф №8590 ЗА ПОСТАВЛЕННЫЙ ТОВАР</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3034,23 +3044,23 @@
           <t>161</t>
         </is>
       </c>
-      <c r="C71" s="2" t="n"/>
-      <c r="D71" s="2" t="n">
-        <v>25783000</v>
-      </c>
+      <c r="C71" s="2" t="n">
+        <v>18761000</v>
+      </c>
+      <c r="D71" s="2" t="n"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Xiva Poligraf MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>345170902</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>20208000851157093001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3060,14 +3070,14 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по договору №20/26, НДС 12%</t>
+          <t>ОПЛАТА ЗА ТОВАРЫ СОГЛАСНО СЧЕТ-ФАКТУРЕ №1878</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>11.08.2026</t>
+          <t>03.08.2026</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3076,39 +3086,39 @@
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>6514000</v>
+        <v>60662000</v>
       </c>
       <c r="D72" s="2" t="n"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №190/26</t>
+          <t>Materiallar uchun oldindan to'lov, shartn. №236/26</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>12.08.2026</t>
+          <t>04.08.2026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3116,40 +3126,40 @@
           <t>163</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
-        <v>10453000</v>
-      </c>
-      <c r="D73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n">
+        <v>10876000</v>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Shodlik Polimer AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>322574503</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>20208000927723213001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Tovarlar uchun to'lov h/f №2204</t>
+          <t>Оплата по счет-фактуре №3658 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>13.08.2026</t>
+          <t>04.08.2026</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3158,39 +3168,34 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>57601000</v>
+        <v>21924000</v>
       </c>
       <c r="D74" s="2" t="n"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>372095842</t>
+          <t>Oqsaroy Bank ATB</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>45994000900000001001</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Materiallar uchun oldindan to'lov, shartnoma №152/26</t>
+          <t>Заработная плата за июль 2026 г. (перечисление на пластиковые карты)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>05.08.2026</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3200,38 +3205,38 @@
       </c>
       <c r="C75" s="2" t="n"/>
       <c r="D75" s="2" t="n">
-        <v>16467000</v>
+        <v>40822000</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Sharq Qurilish MChJ</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>334686280</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000871425759001</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №274 за поставленный товар</t>
+          <t>ОПЛАТА ЗА ПРОДУКЦИЮ ПО ДОГОВОРУ №239/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>14.08.2026</t>
+          <t>05.08.2026</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3239,40 +3244,35 @@
           <t>166</t>
         </is>
       </c>
-      <c r="C76" s="2" t="n"/>
-      <c r="D76" s="2" t="n">
-        <v>2548000</v>
-      </c>
+      <c r="C76" s="2" t="n">
+        <v>62800000</v>
+      </c>
+      <c r="D76" s="2" t="n"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>338466336</t>
+          <t>Kreditni qaytarish hisobvarag'i (L-2025-0233)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>16307000237259787417</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по договору №2/26, НДС 12%</t>
+          <t>Kredit shartnomasi L-2025-0233 bo'yicha navbatdagi to'lov (08.2026)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>06.08.2026</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3280,40 +3280,40 @@
           <t>167</t>
         </is>
       </c>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n">
-        <v>8145000</v>
-      </c>
+      <c r="C77" s="2" t="n">
+        <v>56334000</v>
+      </c>
+      <c r="D77" s="2" t="n"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Qarshi Un Mahsulotlari MChJ</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>278320484</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000799048289001</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №136/26 от 17.08.2026</t>
+          <t>Оплата за транспортные услуги по договору №207/26</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3321,40 +3321,40 @@
           <t>168</t>
         </is>
       </c>
-      <c r="C78" s="2" t="n"/>
-      <c r="D78" s="2" t="n">
-        <v>7599000</v>
-      </c>
+      <c r="C78" s="2" t="n">
+        <v>15906000</v>
+      </c>
+      <c r="D78" s="2" t="n"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Oqtosh Qog'oz AJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>371514300</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>20208000665316781001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №171/26 от 17.08.2026</t>
+          <t>Оплата за товары согласно счет-фактуре №150</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>07.08.2026</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3362,40 +3362,40 @@
           <t>169</t>
         </is>
       </c>
-      <c r="C79" s="2" t="n"/>
-      <c r="D79" s="2" t="n">
-        <v>7270000</v>
-      </c>
+      <c r="C79" s="2" t="n">
+        <v>18150000</v>
+      </c>
+      <c r="D79" s="2" t="n"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Samarqand Qurilish MChJ</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>378388884</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000795834914001</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00987</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №2867 за поставленный товар</t>
+          <t>Оплата за товары согласно с/ф №8881</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>10.08.2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3403,40 +3403,40 @@
           <t>170</t>
         </is>
       </c>
-      <c r="C80" s="2" t="n"/>
-      <c r="D80" s="2" t="n">
-        <v>5217000</v>
-      </c>
+      <c r="C80" s="2" t="n">
+        <v>3465000</v>
+      </c>
+      <c r="D80" s="2" t="n"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Bunyodkor Qurilish MChJ</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>247354122</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000393004688001</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №193/26 от 17.08.2026</t>
+          <t>Bino ijarasi uchun to'lov avgust</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>10.08.2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3444,40 +3444,40 @@
           <t>171</t>
         </is>
       </c>
-      <c r="C81" s="2" t="n"/>
-      <c r="D81" s="2" t="n">
-        <v>2853000</v>
-      </c>
+      <c r="C81" s="2" t="n">
+        <v>10560000</v>
+      </c>
+      <c r="D81" s="2" t="n"/>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kattaqo'rg'on Meva-Sabzavot AJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>281783534</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>20208000647915400001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №204/26 от 17.08.2026</t>
+          <t>Оплата за транспортные услуги по договору №290/26</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>12.08.2026</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3485,40 +3485,40 @@
           <t>172</t>
         </is>
       </c>
-      <c r="C82" s="2" t="n"/>
-      <c r="D82" s="2" t="n">
-        <v>2487000</v>
-      </c>
+      <c r="C82" s="2" t="n">
+        <v>10120000</v>
+      </c>
+      <c r="D82" s="2" t="n"/>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Оплата за продукцию по договору №115/26, НДС 12%</t>
+          <t>Transport xizmatlari uchun to'lov, shartnoma №32/26</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>13.08.2026</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3526,40 +3526,40 @@
           <t>173</t>
         </is>
       </c>
-      <c r="C83" s="2" t="n">
-        <v>2990000</v>
-      </c>
-      <c r="D83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n">
+        <v>10513000</v>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
+          <t>Denov Farm Savdo XK</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>201122905</t>
+          <t>278353466</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>20208000791540008001</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>00987</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Социальный налог за июл 2026 г.</t>
+          <t>Предоплата за товар по договору №232/26 от 13.08.2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>14.08.2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3567,40 +3567,40 @@
           <t>174</t>
         </is>
       </c>
-      <c r="C84" s="2" t="n">
-        <v>2990000</v>
-      </c>
-      <c r="D84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n">
+        <v>14677000</v>
+      </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>201122905</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Налог на доходы физических лиц за июль 2026 г.</t>
+          <t>Оплата за продукцию по договору №142/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>17.08.2026</t>
+          <t>14.08.2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3609,32 +3609,32 @@
         </is>
       </c>
       <c r="C85" s="2" t="n">
-        <v>24418000</v>
+        <v>21327000</v>
       </c>
       <c r="D85" s="2" t="n"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Transport xizmatlari uchun to'lov, shartnoma №40/26</t>
+          <t>Оплата за транспортные услуги по дог. №60/26</t>
         </is>
       </c>
     </row>
@@ -3649,23 +3649,23 @@
           <t>176</t>
         </is>
       </c>
-      <c r="C86" s="2" t="n">
-        <v>66168000</v>
-      </c>
-      <c r="D86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n">
+        <v>89245000</v>
+      </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -3675,14 +3675,14 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Предоплата за материалы по дог. №6/26</t>
+          <t>Предоплата за товар по дог. №38/26 от 17.08.2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3690,40 +3690,40 @@
           <t>177</t>
         </is>
       </c>
-      <c r="C87" s="2" t="n"/>
-      <c r="D87" s="2" t="n">
-        <v>1930000</v>
-      </c>
+      <c r="C87" s="2" t="n">
+        <v>2990000</v>
+      </c>
+      <c r="D87" s="2" t="n"/>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №6935 от 18.08.2026, в т.ч. НДС 12%</t>
+          <t>Iyul oyi uchun ijtimoiy soliq</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>18.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3732,39 +3732,39 @@
         </is>
       </c>
       <c r="C88" s="2" t="n">
-        <v>9847000</v>
+        <v>2990000</v>
       </c>
       <c r="D88" s="2" t="n"/>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №8066</t>
+          <t>Jismoniy shaxslar daromad solig'i iyul 2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>19.08.2026</t>
+          <t>17.08.2026</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3773,39 +3773,39 @@
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>6312000</v>
+        <v>12030000</v>
       </c>
       <c r="D89" s="2" t="n"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Angren Qurilish MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>342103076</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>20208000392529178001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Оплата за упаковочные материалы, с/ф №5678</t>
+          <t>ОПЛАТА ЗА УПАКОВОЧНЫЕ МАТЕРИАЛЫ, С/Ф №4441</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>18.08.2026</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3813,40 +3813,40 @@
           <t>180</t>
         </is>
       </c>
-      <c r="C90" s="2" t="n"/>
-      <c r="D90" s="2" t="n">
-        <v>8878000</v>
-      </c>
+      <c r="C90" s="2" t="n">
+        <v>26142000</v>
+      </c>
+      <c r="D90" s="2" t="n"/>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Oqtosh Qog'oz AJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>371514300</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>20208000665316781001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №6953 от 21.08.2026, в т.ч. НДС 12%</t>
+          <t>Xom ashyo uchun to'lov, shartn. №146/26, QQS bilan</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>19.08.2026</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3856,31 +3856,31 @@
       </c>
       <c r="C91" s="2" t="n"/>
       <c r="D91" s="2" t="n">
-        <v>4027000</v>
+        <v>40705000</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Оплата за товар по с/ф №5410 от 21.08.2026, в т.ч. НДС 12%</t>
+          <t>Tovar uchun to'lov, hisob-faktura №8268 19.08.2026, QQS bilan</t>
         </is>
       </c>
     </row>
@@ -3897,38 +3897,38 @@
       </c>
       <c r="C92" s="2" t="n"/>
       <c r="D92" s="2" t="n">
-        <v>1552000</v>
+        <v>9909000</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №1759 за поставленный товар</t>
+          <t>Оплата по счет-фактуре №8109 за поставленный товар</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>21.08.2026</t>
+          <t>24.08.2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3936,33 +3936,33 @@
           <t>183</t>
         </is>
       </c>
-      <c r="C93" s="2" t="n">
-        <v>5589000</v>
-      </c>
-      <c r="D93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="n">
+        <v>14304000</v>
+      </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>201122905</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>23402000300100001010</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>00014</t>
+          <t>01089</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Qo'shilgan qiymat solig'i iyul oyi</t>
+          <t>Оплата по счет-фактуре №4138 за поставленный товар</t>
         </is>
       </c>
     </row>
@@ -3979,31 +3979,31 @@
       </c>
       <c r="C94" s="2" t="n"/>
       <c r="D94" s="2" t="n">
-        <v>33549000</v>
+        <v>13669000</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Durdona Metall Servis MChJ</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>264917666</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000685036986001</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>01121</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Yetkazilgan tovar uchun to'lov h/f №3567</t>
+          <t>Оплата за продукцию по договору №247/26, НДС 12%</t>
         </is>
       </c>
     </row>
@@ -4018,33 +4018,33 @@
           <t>185</t>
         </is>
       </c>
-      <c r="C95" s="2" t="n"/>
-      <c r="D95" s="2" t="n">
-        <v>5055000</v>
-      </c>
+      <c r="C95" s="2" t="n">
+        <v>2166000</v>
+      </c>
+      <c r="D95" s="2" t="n"/>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Hududiy elektr tarmoqlari AJ</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>200933985</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000028408911001</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Предоплата за товар по дог. №178/26 от 24.08.2026</t>
+          <t>Оплата за электроэнергию за август 2026 г.</t>
         </is>
       </c>
     </row>
@@ -4060,32 +4060,32 @@
         </is>
       </c>
       <c r="C96" s="2" t="n">
-        <v>2166000</v>
+        <v>5944000</v>
       </c>
       <c r="D96" s="2" t="n"/>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Hududiy elektr tarmoqlari AJ</t>
+          <t>Davlat soliq qo'mitasi (budjet hisobvarag'i)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>200933985</t>
+          <t>201122905</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>20208000147014124001</t>
+          <t>23402000300100001010</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>00014</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Оплата за электроэнергию за август 2026 г.</t>
+          <t>Уплата налога на добавленную стоимость за июль</t>
         </is>
       </c>
     </row>
@@ -4101,32 +4101,32 @@
         </is>
       </c>
       <c r="C97" s="2" t="n">
-        <v>7731000</v>
+        <v>12992000</v>
       </c>
       <c r="D97" s="2" t="n"/>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Angren Avto Ehtiyot MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>394504364</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>20208000426795116001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Tovarlar uchun to'lov h/f №2732</t>
+          <t>Оплата за транспортные услуги по договору №2/26</t>
         </is>
       </c>
     </row>
@@ -4143,21 +4143,21 @@
       </c>
       <c r="C98" s="2" t="n"/>
       <c r="D98" s="2" t="n">
-        <v>9682000</v>
+        <v>23677000</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №198/26 от 25.08.2026</t>
+          <t>Оплата по счет-фактуре №5381 за поставленный товар</t>
         </is>
       </c>
     </row>
@@ -4184,21 +4184,21 @@
       </c>
       <c r="C99" s="2" t="n"/>
       <c r="D99" s="2" t="n">
-        <v>5048000</v>
+        <v>18896000</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Оплата по с/ф №2418 за поставленный товар</t>
+          <t>Оплата за товар по счет-фактуре №6038 от 25.08.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
@@ -4223,40 +4223,40 @@
           <t>190</t>
         </is>
       </c>
-      <c r="C100" s="2" t="n"/>
-      <c r="D100" s="2" t="n">
-        <v>2600000</v>
-      </c>
+      <c r="C100" s="2" t="n">
+        <v>8827000</v>
+      </c>
+      <c r="D100" s="2" t="n"/>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>01089</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Предоплата за товар по дог. №292/26 от 25.08.2026</t>
+          <t>TRANSPORT XIZMATLARI UCHUN TO'LOV, SHARTNOMA №104/26</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>25.08.2026</t>
+          <t>26.08.2026</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4266,38 +4266,38 @@
       </c>
       <c r="C101" s="2" t="n"/>
       <c r="D101" s="2" t="n">
-        <v>2546000</v>
+        <v>9647000</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Oydin Avto Savdo AJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>308210196</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>20208000469112014001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Предоплата за товар по договору №128/26 от 25.08.2026</t>
+          <t>Mahsulot uchun to'lov, shartnoma №246/26, QQS 12%</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>25.08.2026</t>
+          <t>26.08.2026</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4306,32 +4306,32 @@
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>9120000</v>
+        <v>9291000</v>
       </c>
       <c r="D102" s="2" t="n"/>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Navro'z Logistik MChJ</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>224447001</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000860836504001</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по дог. №286/26</t>
+          <t>Оплата за упаковочные материалы, с/ф №7315</t>
         </is>
       </c>
     </row>
@@ -4347,32 +4347,32 @@
         </is>
       </c>
       <c r="C103" s="2" t="n">
-        <v>6075000</v>
+        <v>63221000</v>
       </c>
       <c r="D103" s="2" t="n"/>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Farg'ona Qurilish Materiallari MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>213569718</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>20208000980612170001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>01121</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Предоплата за материалы по договору №91/26</t>
+          <t>Оплата за упаковочные материалы, с/ф №4914</t>
         </is>
       </c>
     </row>
@@ -4389,21 +4389,21 @@
       </c>
       <c r="C104" s="2" t="n"/>
       <c r="D104" s="2" t="n">
-        <v>11758000</v>
+        <v>20050000</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Olmaliq Mato MChJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>220649176</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>20208000606850369001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4413,14 +4413,14 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>MAHSULOT UCHUN TO'LOV, SHARTN. №285/26, QQS 12%</t>
+          <t>ОПЛАТА ЗА ПРОДУКЦИЮ ПО ДОГ. №27/26, НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>27.08.2026</t>
+          <t>28.08.2026</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4430,21 +4430,21 @@
       </c>
       <c r="C105" s="2" t="n"/>
       <c r="D105" s="2" t="n">
-        <v>9445000</v>
+        <v>43798000</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Guliston Trans Servis AJ</t>
+          <t>Xiva Mehmonxona MChJ</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>338466336</t>
+          <t>346633682</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>20208000289994840001</t>
+          <t>20208000999484093001</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4454,14 +4454,14 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Предоплата за товар по дог. №26/26 от 27.08.2026</t>
+          <t>Оплата за товар по с/ф №9545 от 28.08.2026, в т.ч. НДС 12%</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>27.08.2026</t>
+          <t>28.08.2026</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4470,22 +4470,22 @@
         </is>
       </c>
       <c r="C106" s="2" t="n">
-        <v>8498000</v>
+        <v>24906000</v>
       </c>
       <c r="D106" s="2" t="n"/>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Samarqand Qurilish MChJ</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>378388884</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000795834914001</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4495,14 +4495,14 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Оплата за сырье по договору №242/26 от 27.08.2026, НДС 12%</t>
+          <t>Оплата за товары согласно счет-фактуре №1623</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>28.08.2026</t>
+          <t>31.08.2026</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4510,33 +4510,33 @@
           <t>197</t>
         </is>
       </c>
-      <c r="C107" s="2" t="n">
-        <v>24882000</v>
-      </c>
-      <c r="D107" s="2" t="n"/>
+      <c r="C107" s="2" t="n"/>
+      <c r="D107" s="2" t="n">
+        <v>27302000</v>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Chust Mehmonxona XK</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>251430036</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000531678108001</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Оплата за транспортные услуги по договору №64/26</t>
+          <t>Оплата за продукцию по договору №220/26, НДС 12%</t>
         </is>
       </c>
     </row>
@@ -4551,33 +4551,28 @@
           <t>198</t>
         </is>
       </c>
-      <c r="C108" s="2" t="n"/>
-      <c r="D108" s="2" t="n">
-        <v>145355000</v>
-      </c>
+      <c r="C108" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D108" s="2" t="n"/>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Farg'ona Poligraf MChJ</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>216346862</t>
+          <t>Oqsaroy Bank ATB</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>20208000098714257001</t>
+          <t>45994000900000001001</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>00962</t>
+          <t>01153</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Оплата по счет-фактуре №9874 за поставленный товар</t>
+          <t>Bank xizmati uchun komissiya</t>
         </is>
       </c>
     </row>
@@ -4592,33 +4587,33 @@
           <t>199</t>
         </is>
       </c>
-      <c r="C109" s="2" t="n"/>
-      <c r="D109" s="2" t="n">
-        <v>4119000</v>
-      </c>
+      <c r="C109" s="2" t="n">
+        <v>8342000</v>
+      </c>
+      <c r="D109" s="2" t="n"/>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Oqtosh Qog'oz AJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>371514300</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>20208000665316781001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Оплата за товар по счет-фактуре №2677 от 31.08.2026, в т.ч. НДС 12%</t>
+          <t>Materiallar uchun oldindan to'lov, shartnoma №18/26</t>
         </is>
       </c>
     </row>
@@ -4634,27 +4629,32 @@
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>300000</v>
+        <v>12410000</v>
       </c>
       <c r="D110" s="2" t="n"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Oqsaroy Bank ATB</t>
+          <t>Chirchiq Sut Mahsulotlari MChJ</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>248779261</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>45994000900000001001</t>
+          <t>20208000881064425001</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>01153</t>
+          <t>01204</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Комиссия банка за расчетно-кассовое обслуживание за август</t>
+          <t>Оплата за товары согласно с/ф №3092</t>
         </is>
       </c>
     </row>
@@ -4670,22 +4670,22 @@
         </is>
       </c>
       <c r="C111" s="2" t="n">
-        <v>13282000</v>
+        <v>16638000</v>
       </c>
       <c r="D111" s="2" t="n"/>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Samarqand Qurilish MChJ</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>378388884</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000795834914001</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Оплата за товары согласно счет-фактуре №8986</t>
+          <t>Оплата за транспортные услуги по договору №216/26</t>
         </is>
       </c>
     </row>
@@ -4711,32 +4711,32 @@
         </is>
       </c>
       <c r="C112" s="2" t="n">
-        <v>20080000</v>
+        <v>17904000</v>
       </c>
       <c r="D112" s="2" t="n"/>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Zarafshon Dori-Darmon MChJ</t>
+          <t>Shodlik Yog' Zavodi MChJ</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>372095842</t>
+          <t>256971819</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>20208000962427631001</t>
+          <t>20208000061217007001</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>00987</t>
+          <t>00962</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Оплата за сырье по договору №163/26 от 31.08.2026, НДС 12%</t>
+          <t>Оплата за сырье по договору №188/26 от 31.08.2026, НДС 12%</t>
         </is>
       </c>
     </row>
@@ -4747,10 +4747,10 @@
         </is>
       </c>
       <c r="C113" s="4" t="n">
-        <v>1005577000</v>
+        <v>1051401000</v>
       </c>
       <c r="D113" s="4" t="n">
-        <v>933977000</v>
+        <v>979801000</v>
       </c>
     </row>
     <row r="114">

</xml_diff>